<commit_message>
Script 1 - atualização automática de dados
</commit_message>
<xml_diff>
--- a/Data/g1.1.xlsx
+++ b/Data/g1.1.xlsx
@@ -453,54 +453,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.28257356816728</v>
+        <v>14.73257689442189</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.38328592034125</v>
+        <v>13.44269577606423</v>
       </c>
       <c r="C3" t="n">
         <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.163532889959003</v>
+        <v>12.88001598426398</v>
       </c>
       <c r="C4" t="n">
         <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
@@ -511,50 +511,50 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.038578912774967</v>
+        <v>7.890383025089162</v>
       </c>
       <c r="C5" t="n">
         <v>4</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AC</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5.979340654464274</v>
+        <v>5.652659822157795</v>
       </c>
       <c r="C6" t="n">
         <v>5</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5.639044878530812</v>
+        <v>4.816953216278661</v>
       </c>
       <c r="C7" t="n">
         <v>6</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
@@ -565,14 +565,14 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1.251393607016045</v>
+        <v>3.118144130554446</v>
       </c>
       <c r="C8" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
@@ -583,12 +583,12 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.016694345902016</v>
+        <v>3.241657824791806</v>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
@@ -599,48 +599,48 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3.554673531071183</v>
+        <v>2.867008788862638</v>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Variação (%) 2022</t>
+          <t>Variação (%) 2023</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>57.303631404687</v>
+        <v>77.14346626765018</v>
       </c>
       <c r="C11" t="n">
         <v>1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>56.93075937581798</v>
+        <v>63.84407511155798</v>
       </c>
       <c r="C12" t="n">
         <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
@@ -651,68 +651,68 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>47.69781593734575</v>
+        <v>59.35173933449352</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>32.6068937425523</v>
+        <v>49.57179111911111</v>
       </c>
       <c r="C14" t="n">
         <v>4</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>31.84788151928765</v>
+        <v>42.69524774665621</v>
       </c>
       <c r="C15" t="n">
         <v>5</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>29.69759694720014</v>
+        <v>36.70681689547283</v>
       </c>
       <c r="C16" t="n">
         <v>6</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
@@ -723,14 +723,14 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4.078908858016646</v>
+        <v>7.324239245718005</v>
       </c>
       <c r="C17" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
@@ -741,12 +741,12 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11.52892348592597</v>
+        <v>15.14430956101356</v>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>
@@ -757,12 +757,12 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>13.60673175406315</v>
+        <v>16.86384673819174</v>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Variação (%) 2022/2010</t>
+          <t>Variação (%) 2023/2010</t>
         </is>
       </c>
     </row>

</xml_diff>